<commit_message>
Orders workbook: add Weekly Watch sheet (watch log + paper mark-to-market)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BBnnwzPLx94vYYG3d4vP48
</commit_message>
<xml_diff>
--- a/RotationOrders.xlsx
+++ b/RotationOrders.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="Orders" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Data" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Weekly Watch" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,11 +18,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="$#,##0"/>
     <numFmt numFmtId="165" formatCode="$#,##0;($#,##0);-"/>
+    <numFmt numFmtId="166" formatCode="+0.0%;-0.0%"/>
+    <numFmt numFmtId="167" formatCode="+0.00%;-0.00%"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -82,6 +85,12 @@
       <color rgb="00000000"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="001F3864"/>
+      <sz val="12"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -132,7 +141,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -161,6 +170,9 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1270,4 +1282,303 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="001F3864"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="22" t="inlineStr">
+        <is>
+          <t>WEEKLY REGIME WATCH — informational, trades nothing</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="8" t="inlineStr">
+        <is>
+          <t>Distance of each price to its regime boundary (mean of the prior 9 completed monthly closes). Provisional = quadrant if the month ended that day. Only the monthly ledger row rotates money (TESTS.md entry 67).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>Date (UTC)</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>SPY vs growth line</t>
+        </is>
+      </c>
+      <c r="C4" s="9" t="inlineStr">
+        <is>
+          <t>DBC vs inflation line</t>
+        </is>
+      </c>
+      <c r="D4" s="9" t="inlineStr">
+        <is>
+          <t>Provisional</t>
+        </is>
+      </c>
+      <c r="E4" s="9" t="inlineStr">
+        <is>
+          <t>In force</t>
+        </is>
+      </c>
+      <c r="F4" s="9" t="inlineStr">
+        <is>
+          <t>Divergence</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B5" s="23" t="n">
+        <v>0.07099999999999999</v>
+      </c>
+      <c r="C5" s="23" t="n">
+        <v>0.1549</v>
+      </c>
+      <c r="D5" s="13" t="inlineStr">
+        <is>
+          <t>REFLATION</t>
+        </is>
+      </c>
+      <c r="E5" s="13" t="inlineStr">
+        <is>
+          <t>REFLATION</t>
+        </is>
+      </c>
+      <c r="F5" s="13" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B6" s="23" t="n">
+        <v>0.0698</v>
+      </c>
+      <c r="C6" s="23" t="n">
+        <v>0.1994</v>
+      </c>
+      <c r="D6" s="13" t="inlineStr">
+        <is>
+          <t>REFLATION</t>
+        </is>
+      </c>
+      <c r="E6" s="13" t="inlineStr">
+        <is>
+          <t>REFLATION</t>
+        </is>
+      </c>
+      <c r="F6" s="13" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B7" s="23" t="n">
+        <v>0.0688</v>
+      </c>
+      <c r="C7" s="23" t="n">
+        <v>0.1911</v>
+      </c>
+      <c r="D7" s="13" t="inlineStr">
+        <is>
+          <t>REFLATION</t>
+        </is>
+      </c>
+      <c r="E7" s="13" t="inlineStr">
+        <is>
+          <t>REFLATION</t>
+        </is>
+      </c>
+      <c r="F7" s="13" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Paper ledger mark-to-market (as of 2026-09-21)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>Tier</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>Since</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>Return</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>Max drawdown</t>
+        </is>
+      </c>
+      <c r="E11" s="9" t="inlineStr">
+        <is>
+          <t>Trading days</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="13" t="inlineStr">
+        <is>
+          <t>CONS</t>
+        </is>
+      </c>
+      <c r="B12" s="13" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="C12" s="24" t="n">
+        <v>-0.0006219471265683785</v>
+      </c>
+      <c r="D12" s="24" t="n">
+        <v>-0.01038263314449761</v>
+      </c>
+      <c r="E12" s="13" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="13" t="inlineStr">
+        <is>
+          <t>MOD</t>
+        </is>
+      </c>
+      <c r="B13" s="13" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="C13" s="24" t="n">
+        <v>0.001452225303145926</v>
+      </c>
+      <c r="D13" s="24" t="n">
+        <v>-0.01483572557923674</v>
+      </c>
+      <c r="E13" s="13" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="13" t="inlineStr">
+        <is>
+          <t>AGG</t>
+        </is>
+      </c>
+      <c r="B14" s="13" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="C14" s="24" t="n">
+        <v>0.01534823114767803</v>
+      </c>
+      <c r="D14" s="24" t="n">
+        <v>-0.02194480807823074</v>
+      </c>
+      <c r="E14" s="13" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="13" t="inlineStr">
+        <is>
+          <t>VAGG</t>
+        </is>
+      </c>
+      <c r="B15" s="13" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="C15" s="24" t="n">
+        <v>0.0167725625138937</v>
+      </c>
+      <c r="D15" s="24" t="n">
+        <v>-0.03546264636746566</v>
+      </c>
+      <c r="E15" s="13" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="13" t="inlineStr">
+        <is>
+          <t>SPY (bench)</t>
+        </is>
+      </c>
+      <c r="B16" s="13" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="C16" s="24" t="n">
+        <v>0.01151419157187794</v>
+      </c>
+      <c r="D16" s="24" t="n">
+        <v>-0.02472935182691627</v>
+      </c>
+      <c r="E16" s="13" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>Daily-rebalanced paper books from each ledger row's logged_at; SPY = buy-and-hold benchmark.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Order workbook: --provisional next-month preview (ledger untouched); October provisional build
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BBnnwzPLx94vYYG3d4vP48
</commit_message>
<xml_diff>
--- a/RotationOrders.xlsx
+++ b/RotationOrders.xlsx
@@ -1064,7 +1064,7 @@
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>2026-09</t>
+          <t>2026-10</t>
         </is>
       </c>
     </row>
@@ -1104,7 +1104,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>v8 (restated from logged signals)</t>
+          <t>v8 — PROVISIONAL intraday Sept 30, 2:35pm ET (ledger row not yet logged)</t>
         </is>
       </c>
     </row>
@@ -1209,7 +1209,7 @@
         </is>
       </c>
       <c r="B23" s="21" t="n">
-        <v>0.315</v>
+        <v>0.2275</v>
       </c>
     </row>
     <row r="24">
@@ -1229,7 +1229,7 @@
         </is>
       </c>
       <c r="B25" s="21" t="n">
-        <v>0.2275</v>
+        <v>0.315</v>
       </c>
     </row>
     <row r="31">
@@ -1256,7 +1256,7 @@
         </is>
       </c>
       <c r="B33" s="21" t="n">
-        <v>0.315</v>
+        <v>0.2275</v>
       </c>
     </row>
     <row r="34">
@@ -1276,7 +1276,7 @@
         </is>
       </c>
       <c r="B35" s="21" t="n">
-        <v>0.2275</v>
+        <v>0.315</v>
       </c>
     </row>
   </sheetData>
@@ -1291,7 +1291,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1432,65 +1432,72 @@
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>Paper ledger mark-to-market (as of 2026-09-21)</t>
+    <row r="8">
+      <c r="A8" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B8" s="23" t="n">
+        <v>0.0723</v>
+      </c>
+      <c r="C8" s="23" t="n">
+        <v>0.1574</v>
+      </c>
+      <c r="D8" s="13" t="inlineStr">
+        <is>
+          <t>REFLATION</t>
+        </is>
+      </c>
+      <c r="E8" s="13" t="inlineStr">
+        <is>
+          <t>REFLATION</t>
+        </is>
+      </c>
+      <c r="F8" s="13" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="9" t="inlineStr">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Paper ledger mark-to-market (as of 2026-09-30)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="inlineStr">
         <is>
           <t>Tier</t>
         </is>
       </c>
-      <c r="B11" s="9" t="inlineStr">
+      <c r="B12" s="9" t="inlineStr">
         <is>
           <t>Since</t>
         </is>
       </c>
-      <c r="C11" s="9" t="inlineStr">
+      <c r="C12" s="9" t="inlineStr">
         <is>
           <t>Return</t>
         </is>
       </c>
-      <c r="D11" s="9" t="inlineStr">
+      <c r="D12" s="9" t="inlineStr">
         <is>
           <t>Max drawdown</t>
         </is>
       </c>
-      <c r="E11" s="9" t="inlineStr">
+      <c r="E12" s="9" t="inlineStr">
         <is>
           <t>Trading days</t>
         </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="13" t="inlineStr">
-        <is>
-          <t>CONS</t>
-        </is>
-      </c>
-      <c r="B12" s="13" t="inlineStr">
-        <is>
-          <t>2026-08-20</t>
-        </is>
-      </c>
-      <c r="C12" s="24" t="n">
-        <v>-0.0006219471265683785</v>
-      </c>
-      <c r="D12" s="24" t="n">
-        <v>-0.01038263314449761</v>
-      </c>
-      <c r="E12" s="13" t="n">
-        <v>21</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="13" t="inlineStr">
         <is>
-          <t>MOD</t>
+          <t>CONS</t>
         </is>
       </c>
       <c r="B13" s="13" t="inlineStr">
@@ -1499,19 +1506,19 @@
         </is>
       </c>
       <c r="C13" s="24" t="n">
-        <v>0.001452225303145926</v>
+        <v>-0.008831455100244301</v>
       </c>
       <c r="D13" s="24" t="n">
-        <v>-0.01483572557923674</v>
+        <v>-0.02204983834410612</v>
       </c>
       <c r="E13" s="13" t="n">
-        <v>21</v>
+        <v>28</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="13" t="inlineStr">
         <is>
-          <t>AGG</t>
+          <t>MOD</t>
         </is>
       </c>
       <c r="B14" s="13" t="inlineStr">
@@ -1520,19 +1527,19 @@
         </is>
       </c>
       <c r="C14" s="24" t="n">
-        <v>0.01534823114767803</v>
+        <v>-0.009661122072122885</v>
       </c>
       <c r="D14" s="24" t="n">
-        <v>-0.02194480807823074</v>
+        <v>-0.03063726832854285</v>
       </c>
       <c r="E14" s="13" t="n">
-        <v>21</v>
+        <v>28</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="13" t="inlineStr">
         <is>
-          <t>VAGG</t>
+          <t>AGG</t>
         </is>
       </c>
       <c r="B15" s="13" t="inlineStr">
@@ -1541,38 +1548,59 @@
         </is>
       </c>
       <c r="C15" s="24" t="n">
-        <v>0.0167725625138937</v>
+        <v>0.007714972641025941</v>
       </c>
       <c r="D15" s="24" t="n">
-        <v>-0.03546264636746566</v>
+        <v>-0.02704464641821624</v>
       </c>
       <c r="E15" s="13" t="n">
-        <v>21</v>
+        <v>28</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="13" t="inlineStr">
         <is>
+          <t>VAGG</t>
+        </is>
+      </c>
+      <c r="B16" s="13" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="C16" s="24" t="n">
+        <v>0.005172306469189758</v>
+      </c>
+      <c r="D16" s="24" t="n">
+        <v>-0.03546264302986191</v>
+      </c>
+      <c r="E16" s="13" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="13" t="inlineStr">
+        <is>
           <t>SPY (bench)</t>
         </is>
       </c>
-      <c r="B16" s="13" t="inlineStr">
+      <c r="B17" s="13" t="inlineStr">
         <is>
           <t>2026-08-20</t>
         </is>
       </c>
-      <c r="C16" s="24" t="n">
-        <v>0.01151419157187794</v>
-      </c>
-      <c r="D16" s="24" t="n">
+      <c r="C17" s="24" t="n">
+        <v>0.007268189509373579</v>
+      </c>
+      <c r="D17" s="24" t="n">
         <v>-0.02472935182691627</v>
       </c>
-      <c r="E16" s="13" t="n">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="8" t="inlineStr">
+      <c r="E17" s="13" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="8" t="inlineStr">
         <is>
           <t>Daily-rebalanced paper books from each ledger row's logged_at; SPY = buy-and-hold benchmark.</t>
         </is>

</xml_diff>

<commit_message>
October order sheet on final Sept 30 closes (provisional until the Oct 1 ledger row)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BBnnwzPLx94vYYG3d4vP48
</commit_message>
<xml_diff>
--- a/RotationOrders.xlsx
+++ b/RotationOrders.xlsx
@@ -1104,7 +1104,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>v8 — PROVISIONAL intraday Sept 30, 2:35pm ET (ledger row not yet logged)</t>
+          <t>v8 — PROVISIONAL final Sept 30 closes; ledger row logs Oct 1 (ledger row not yet logged)</t>
         </is>
       </c>
     </row>
@@ -1506,7 +1506,7 @@
         </is>
       </c>
       <c r="C13" s="24" t="n">
-        <v>-0.008831455100244301</v>
+        <v>-0.01123286072329011</v>
       </c>
       <c r="D13" s="24" t="n">
         <v>-0.02204983834410612</v>
@@ -1527,7 +1527,7 @@
         </is>
       </c>
       <c r="C14" s="24" t="n">
-        <v>-0.009661122072122885</v>
+        <v>-0.01314860542558849</v>
       </c>
       <c r="D14" s="24" t="n">
         <v>-0.03063726832854285</v>
@@ -1548,7 +1548,7 @@
         </is>
       </c>
       <c r="C15" s="24" t="n">
-        <v>0.007714972641025941</v>
+        <v>0.00244083712240073</v>
       </c>
       <c r="D15" s="24" t="n">
         <v>-0.02704464641821624</v>
@@ -1569,7 +1569,7 @@
         </is>
       </c>
       <c r="C16" s="24" t="n">
-        <v>0.005172306469189758</v>
+        <v>-0.004121304920642221</v>
       </c>
       <c r="D16" s="24" t="n">
         <v>-0.03546264302986191</v>
@@ -1590,7 +1590,7 @@
         </is>
       </c>
       <c r="C17" s="24" t="n">
-        <v>0.007268189509373579</v>
+        <v>0.002325432308721398</v>
       </c>
       <c r="D17" s="24" t="n">
         <v>-0.02472935182691627</v>

</xml_diff>

<commit_message>
Paper log: 2026-10 row (first under matrix v8); month-start watch; October order sheet
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BBnnwzPLx94vYYG3d4vP48
</commit_message>
<xml_diff>
--- a/RotationOrders.xlsx
+++ b/RotationOrders.xlsx
@@ -1104,7 +1104,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>v8 — PROVISIONAL final Sept 30 closes; ledger row logs Oct 1 (ledger row not yet logged)</t>
+          <t>v8</t>
         </is>
       </c>
     </row>
@@ -1291,7 +1291,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1460,65 +1460,72 @@
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>Paper ledger mark-to-market (as of 2026-09-30)</t>
+    <row r="9">
+      <c r="A9" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B9" s="23" t="n">
+        <v>0.056</v>
+      </c>
+      <c r="C9" s="23" t="n">
+        <v>0.124</v>
+      </c>
+      <c r="D9" s="13" t="inlineStr">
+        <is>
+          <t>REFLATION</t>
+        </is>
+      </c>
+      <c r="E9" s="13" t="inlineStr">
+        <is>
+          <t>REFLATION</t>
+        </is>
+      </c>
+      <c r="F9" s="13" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="9" t="inlineStr">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Paper ledger mark-to-market (as of 2026-10-01)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr">
         <is>
           <t>Tier</t>
         </is>
       </c>
-      <c r="B12" s="9" t="inlineStr">
+      <c r="B13" s="9" t="inlineStr">
         <is>
           <t>Since</t>
         </is>
       </c>
-      <c r="C12" s="9" t="inlineStr">
+      <c r="C13" s="9" t="inlineStr">
         <is>
           <t>Return</t>
         </is>
       </c>
-      <c r="D12" s="9" t="inlineStr">
+      <c r="D13" s="9" t="inlineStr">
         <is>
           <t>Max drawdown</t>
         </is>
       </c>
-      <c r="E12" s="9" t="inlineStr">
+      <c r="E13" s="9" t="inlineStr">
         <is>
           <t>Trading days</t>
         </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="13" t="inlineStr">
-        <is>
-          <t>CONS</t>
-        </is>
-      </c>
-      <c r="B13" s="13" t="inlineStr">
-        <is>
-          <t>2026-08-20</t>
-        </is>
-      </c>
-      <c r="C13" s="24" t="n">
-        <v>-0.01123286072329011</v>
-      </c>
-      <c r="D13" s="24" t="n">
-        <v>-0.02204983834410612</v>
-      </c>
-      <c r="E13" s="13" t="n">
-        <v>28</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="13" t="inlineStr">
         <is>
-          <t>MOD</t>
+          <t>CONS</t>
         </is>
       </c>
       <c r="B14" s="13" t="inlineStr">
@@ -1527,19 +1534,19 @@
         </is>
       </c>
       <c r="C14" s="24" t="n">
-        <v>-0.01314860542558849</v>
+        <v>-0.01075076165774635</v>
       </c>
       <c r="D14" s="24" t="n">
-        <v>-0.03063726832854285</v>
+        <v>-0.02204983834410612</v>
       </c>
       <c r="E14" s="13" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="13" t="inlineStr">
         <is>
-          <t>AGG</t>
+          <t>MOD</t>
         </is>
       </c>
       <c r="B15" s="13" t="inlineStr">
@@ -1548,19 +1555,19 @@
         </is>
       </c>
       <c r="C15" s="24" t="n">
-        <v>0.00244083712240073</v>
+        <v>-0.01128953289984524</v>
       </c>
       <c r="D15" s="24" t="n">
-        <v>-0.02704464641821624</v>
+        <v>-0.03063726832854285</v>
       </c>
       <c r="E15" s="13" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="13" t="inlineStr">
         <is>
-          <t>VAGG</t>
+          <t>AGG</t>
         </is>
       </c>
       <c r="B16" s="13" t="inlineStr">
@@ -1569,38 +1576,59 @@
         </is>
       </c>
       <c r="C16" s="24" t="n">
-        <v>-0.004121304920642221</v>
+        <v>0.0031102273129191</v>
       </c>
       <c r="D16" s="24" t="n">
-        <v>-0.03546264302986191</v>
+        <v>-0.02704464641821624</v>
       </c>
       <c r="E16" s="13" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="13" t="inlineStr">
         <is>
+          <t>VAGG</t>
+        </is>
+      </c>
+      <c r="B17" s="13" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="C17" s="24" t="n">
+        <v>-0.003106967803359173</v>
+      </c>
+      <c r="D17" s="24" t="n">
+        <v>-0.03546264302986191</v>
+      </c>
+      <c r="E17" s="13" t="n">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="13" t="inlineStr">
+        <is>
           <t>SPY (bench)</t>
         </is>
       </c>
-      <c r="B17" s="13" t="inlineStr">
+      <c r="B18" s="13" t="inlineStr">
         <is>
           <t>2026-08-20</t>
         </is>
       </c>
-      <c r="C17" s="24" t="n">
-        <v>0.002325432308721398</v>
-      </c>
-      <c r="D17" s="24" t="n">
+      <c r="C18" s="24" t="n">
+        <v>0.0008071576105210809</v>
+      </c>
+      <c r="D18" s="24" t="n">
         <v>-0.02472935182691627</v>
       </c>
-      <c r="E17" s="13" t="n">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="8" t="inlineStr">
+      <c r="E18" s="13" t="n">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="8" t="inlineStr">
         <is>
           <t>Daily-rebalanced paper books from each ledger row's logged_at; SPY = buy-and-hold benchmark.</t>
         </is>

</xml_diff>

<commit_message>
v9 official stats (in-repo), GrowthProjection.xlsx updated in place, October order sheet restated under v9
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BBnnwzPLx94vYYG3d4vP48
</commit_message>
<xml_diff>
--- a/RotationOrders.xlsx
+++ b/RotationOrders.xlsx
@@ -749,7 +749,7 @@
     <row r="14">
       <c r="A14" s="10" t="inlineStr">
         <is>
-          <t>GDX</t>
+          <t>GLD</t>
         </is>
       </c>
       <c r="B14" s="11" t="n">
@@ -1104,7 +1104,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>v8</t>
+          <t>v9 (restated from logged signals)</t>
         </is>
       </c>
     </row>
@@ -1215,7 +1215,7 @@
     <row r="24">
       <c r="A24" s="19" t="inlineStr">
         <is>
-          <t>GDX</t>
+          <t>GLD</t>
         </is>
       </c>
       <c r="B24" s="21" t="n">
@@ -1262,7 +1262,7 @@
     <row r="34">
       <c r="A34" s="19" t="inlineStr">
         <is>
-          <t>GDX</t>
+          <t>GLD</t>
         </is>
       </c>
       <c r="B34" s="21" t="n">
@@ -1291,7 +1291,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1488,65 +1488,72 @@
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>Paper ledger mark-to-market (as of 2026-10-01)</t>
+    <row r="10">
+      <c r="A10" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B10" s="23" t="n">
+        <v>0.06569999999999999</v>
+      </c>
+      <c r="C10" s="23" t="n">
+        <v>0.1317</v>
+      </c>
+      <c r="D10" s="13" t="inlineStr">
+        <is>
+          <t>REFLATION</t>
+        </is>
+      </c>
+      <c r="E10" s="13" t="inlineStr">
+        <is>
+          <t>REFLATION</t>
+        </is>
+      </c>
+      <c r="F10" s="13" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="9" t="inlineStr">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Paper ledger mark-to-market (as of 2026-10-08)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
         <is>
           <t>Tier</t>
         </is>
       </c>
-      <c r="B13" s="9" t="inlineStr">
+      <c r="B14" s="9" t="inlineStr">
         <is>
           <t>Since</t>
         </is>
       </c>
-      <c r="C13" s="9" t="inlineStr">
+      <c r="C14" s="9" t="inlineStr">
         <is>
           <t>Return</t>
         </is>
       </c>
-      <c r="D13" s="9" t="inlineStr">
+      <c r="D14" s="9" t="inlineStr">
         <is>
           <t>Max drawdown</t>
         </is>
       </c>
-      <c r="E13" s="9" t="inlineStr">
+      <c r="E14" s="9" t="inlineStr">
         <is>
           <t>Trading days</t>
         </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="13" t="inlineStr">
-        <is>
-          <t>CONS</t>
-        </is>
-      </c>
-      <c r="B14" s="13" t="inlineStr">
-        <is>
-          <t>2026-08-20</t>
-        </is>
-      </c>
-      <c r="C14" s="24" t="n">
-        <v>-0.01075076165774635</v>
-      </c>
-      <c r="D14" s="24" t="n">
-        <v>-0.02204983834410612</v>
-      </c>
-      <c r="E14" s="13" t="n">
-        <v>29</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="13" t="inlineStr">
         <is>
-          <t>MOD</t>
+          <t>CONS</t>
         </is>
       </c>
       <c r="B15" s="13" t="inlineStr">
@@ -1555,19 +1562,19 @@
         </is>
       </c>
       <c r="C15" s="24" t="n">
-        <v>-0.01128953289984524</v>
+        <v>0.005435441437535493</v>
       </c>
       <c r="D15" s="24" t="n">
-        <v>-0.03063726832854285</v>
+        <v>-0.02204984823786937</v>
       </c>
       <c r="E15" s="13" t="n">
-        <v>29</v>
+        <v>34</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="13" t="inlineStr">
         <is>
-          <t>AGG</t>
+          <t>MOD</t>
         </is>
       </c>
       <c r="B16" s="13" t="inlineStr">
@@ -1576,19 +1583,19 @@
         </is>
       </c>
       <c r="C16" s="24" t="n">
-        <v>0.0031102273129191</v>
+        <v>0.00971772608968946</v>
       </c>
       <c r="D16" s="24" t="n">
-        <v>-0.02704464641821624</v>
+        <v>-0.03063726832854285</v>
       </c>
       <c r="E16" s="13" t="n">
-        <v>29</v>
+        <v>34</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="13" t="inlineStr">
         <is>
-          <t>VAGG</t>
+          <t>AGG</t>
         </is>
       </c>
       <c r="B17" s="13" t="inlineStr">
@@ -1597,38 +1604,59 @@
         </is>
       </c>
       <c r="C17" s="24" t="n">
-        <v>-0.003106967803359173</v>
+        <v>0.03400545200224259</v>
       </c>
       <c r="D17" s="24" t="n">
-        <v>-0.03546264302986191</v>
+        <v>-0.02704464641821624</v>
       </c>
       <c r="E17" s="13" t="n">
-        <v>29</v>
+        <v>34</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="13" t="inlineStr">
         <is>
+          <t>VAGG</t>
+        </is>
+      </c>
+      <c r="B18" s="13" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="C18" s="24" t="n">
+        <v>0.04318087167039097</v>
+      </c>
+      <c r="D18" s="24" t="n">
+        <v>-0.03546264302986191</v>
+      </c>
+      <c r="E18" s="13" t="n">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="13" t="inlineStr">
+        <is>
           <t>SPY (bench)</t>
         </is>
       </c>
-      <c r="B18" s="13" t="inlineStr">
+      <c r="B19" s="13" t="inlineStr">
         <is>
           <t>2026-08-20</t>
         </is>
       </c>
-      <c r="C18" s="24" t="n">
-        <v>0.0008071576105210809</v>
-      </c>
-      <c r="D18" s="24" t="n">
+      <c r="C19" s="24" t="n">
+        <v>0.02003917201675987</v>
+      </c>
+      <c r="D19" s="24" t="n">
         <v>-0.02472935182691627</v>
       </c>
-      <c r="E18" s="13" t="n">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="8" t="inlineStr">
+      <c r="E19" s="13" t="n">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="8" t="inlineStr">
         <is>
           <t>Daily-rebalanced paper books from each ledger row's logged_at; SPY = buy-and-hold benchmark.</t>
         </is>

</xml_diff>

<commit_message>
Orders workbook: --equity option; regenerated at $17,500 (AGG, v9 October book)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BBnnwzPLx94vYYG3d4vP48
</commit_message>
<xml_diff>
--- a/RotationOrders.xlsx
+++ b/RotationOrders.xlsx
@@ -602,7 +602,7 @@
         </is>
       </c>
       <c r="C6" s="7" t="n">
-        <v>11000</v>
+        <v>17500</v>
       </c>
     </row>
     <row r="7">
@@ -1291,7 +1291,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F20"/>
+  <dimension ref="A1:F23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1516,107 +1516,128 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B11" s="23" t="n">
+        <v>0.078</v>
+      </c>
+      <c r="C11" s="23" t="n">
+        <v>0.1463</v>
+      </c>
+      <c r="D11" s="13" t="inlineStr">
+        <is>
+          <t>REFLATION</t>
+        </is>
+      </c>
+      <c r="E11" s="13" t="inlineStr">
+        <is>
+          <t>REFLATION</t>
+        </is>
+      </c>
+      <c r="F11" s="13" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B12" s="23" t="n">
+        <v>0.0568</v>
+      </c>
+      <c r="C12" s="23" t="n">
+        <v>0.1734</v>
+      </c>
+      <c r="D12" s="13" t="inlineStr">
+        <is>
+          <t>REFLATION</t>
+        </is>
+      </c>
+      <c r="E12" s="13" t="inlineStr">
+        <is>
+          <t>REFLATION</t>
+        </is>
+      </c>
+      <c r="F12" s="13" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
     <row r="13">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>Paper ledger mark-to-market (as of 2026-10-08)</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="9" t="inlineStr">
+      <c r="A13" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B13" s="23" t="n">
+        <v>0.0523</v>
+      </c>
+      <c r="C13" s="23" t="n">
+        <v>0.1859</v>
+      </c>
+      <c r="D13" s="13" t="inlineStr">
+        <is>
+          <t>REFLATION</t>
+        </is>
+      </c>
+      <c r="E13" s="13" t="inlineStr">
+        <is>
+          <t>REFLATION</t>
+        </is>
+      </c>
+      <c r="F13" s="13" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Paper ledger mark-to-market (as of 2026-10-24)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="9" t="inlineStr">
         <is>
           <t>Tier</t>
         </is>
       </c>
-      <c r="B14" s="9" t="inlineStr">
+      <c r="B17" s="9" t="inlineStr">
         <is>
           <t>Since</t>
         </is>
       </c>
-      <c r="C14" s="9" t="inlineStr">
+      <c r="C17" s="9" t="inlineStr">
         <is>
           <t>Return</t>
         </is>
       </c>
-      <c r="D14" s="9" t="inlineStr">
+      <c r="D17" s="9" t="inlineStr">
         <is>
           <t>Max drawdown</t>
         </is>
       </c>
-      <c r="E14" s="9" t="inlineStr">
+      <c r="E17" s="9" t="inlineStr">
         <is>
           <t>Trading days</t>
         </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="13" t="inlineStr">
-        <is>
-          <t>CONS</t>
-        </is>
-      </c>
-      <c r="B15" s="13" t="inlineStr">
-        <is>
-          <t>2026-08-20</t>
-        </is>
-      </c>
-      <c r="C15" s="24" t="n">
-        <v>0.005435441437535493</v>
-      </c>
-      <c r="D15" s="24" t="n">
-        <v>-0.02204984823786937</v>
-      </c>
-      <c r="E15" s="13" t="n">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="13" t="inlineStr">
-        <is>
-          <t>MOD</t>
-        </is>
-      </c>
-      <c r="B16" s="13" t="inlineStr">
-        <is>
-          <t>2026-08-20</t>
-        </is>
-      </c>
-      <c r="C16" s="24" t="n">
-        <v>0.00971772608968946</v>
-      </c>
-      <c r="D16" s="24" t="n">
-        <v>-0.03063726832854285</v>
-      </c>
-      <c r="E16" s="13" t="n">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="13" t="inlineStr">
-        <is>
-          <t>AGG</t>
-        </is>
-      </c>
-      <c r="B17" s="13" t="inlineStr">
-        <is>
-          <t>2026-08-20</t>
-        </is>
-      </c>
-      <c r="C17" s="24" t="n">
-        <v>0.03400545200224259</v>
-      </c>
-      <c r="D17" s="24" t="n">
-        <v>-0.02704464641821624</v>
-      </c>
-      <c r="E17" s="13" t="n">
-        <v>34</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="13" t="inlineStr">
         <is>
-          <t>VAGG</t>
+          <t>CONS</t>
         </is>
       </c>
       <c r="B18" s="13" t="inlineStr">
@@ -1625,38 +1646,101 @@
         </is>
       </c>
       <c r="C18" s="24" t="n">
-        <v>0.04318087167039097</v>
+        <v>0.01732079494266392</v>
       </c>
       <c r="D18" s="24" t="n">
-        <v>-0.03546264302986191</v>
+        <v>-0.02204984823786937</v>
       </c>
       <c r="E18" s="13" t="n">
-        <v>34</v>
+        <v>45</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="13" t="inlineStr">
         <is>
+          <t>MOD</t>
+        </is>
+      </c>
+      <c r="B19" s="13" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="C19" s="24" t="n">
+        <v>0.02478359698872024</v>
+      </c>
+      <c r="D19" s="24" t="n">
+        <v>-0.03063726832854285</v>
+      </c>
+      <c r="E19" s="13" t="n">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="13" t="inlineStr">
+        <is>
+          <t>AGG</t>
+        </is>
+      </c>
+      <c r="B20" s="13" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="C20" s="24" t="n">
+        <v>0.04366982008972542</v>
+      </c>
+      <c r="D20" s="24" t="n">
+        <v>-0.02704464641821624</v>
+      </c>
+      <c r="E20" s="13" t="n">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="13" t="inlineStr">
+        <is>
+          <t>VAGG</t>
+        </is>
+      </c>
+      <c r="B21" s="13" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="C21" s="24" t="n">
+        <v>0.008901791907482304</v>
+      </c>
+      <c r="D21" s="24" t="n">
+        <v>-0.05516467405412073</v>
+      </c>
+      <c r="E21" s="13" t="n">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="13" t="inlineStr">
+        <is>
           <t>SPY (bench)</t>
         </is>
       </c>
-      <c r="B19" s="13" t="inlineStr">
+      <c r="B22" s="13" t="inlineStr">
         <is>
           <t>2026-08-20</t>
         </is>
       </c>
-      <c r="C19" s="24" t="n">
-        <v>0.02003917201675987</v>
-      </c>
-      <c r="D19" s="24" t="n">
+      <c r="C22" s="24" t="n">
+        <v>-0.0009741253031163577</v>
+      </c>
+      <c r="D22" s="24" t="n">
         <v>-0.02472935182691627</v>
       </c>
-      <c r="E19" s="13" t="n">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="8" t="inlineStr">
+      <c r="E22" s="13" t="n">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="8" t="inlineStr">
         <is>
           <t>Daily-rebalanced paper books from each ledger row's logged_at; SPY = buy-and-hold benchmark.</t>
         </is>

</xml_diff>

<commit_message>
Order sheet on the November book (final Oct closes, provisional until the Nov 1 row), $17,500
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BBnnwzPLx94vYYG3d4vP48
</commit_message>
<xml_diff>
--- a/RotationOrders.xlsx
+++ b/RotationOrders.xlsx
@@ -1064,7 +1064,7 @@
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>2026-10</t>
+          <t>2026-11</t>
         </is>
       </c>
     </row>
@@ -1095,7 +1095,7 @@
         </is>
       </c>
       <c r="B3" s="21" t="n">
-        <v>0.1593</v>
+        <v>0.2205</v>
       </c>
       <c r="G3" s="20" t="inlineStr">
         <is>
@@ -1104,7 +1104,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>v9 (restated from logged signals)</t>
+          <t>v9 — PROVISIONAL final Oct 30 closes; ledger row logs Nov 1 (ledger row not yet logged)</t>
         </is>
       </c>
     </row>
@@ -1125,7 +1125,7 @@
         </is>
       </c>
       <c r="B5" s="21" t="n">
-        <v>0.2205</v>
+        <v>0.1593</v>
       </c>
     </row>
     <row r="6">
@@ -1162,7 +1162,7 @@
         </is>
       </c>
       <c r="B13" s="21" t="n">
-        <v>0.2275</v>
+        <v>0.315</v>
       </c>
     </row>
     <row r="14">
@@ -1182,7 +1182,7 @@
         </is>
       </c>
       <c r="B15" s="21" t="n">
-        <v>0.315</v>
+        <v>0.2275</v>
       </c>
     </row>
     <row r="21">
@@ -1209,7 +1209,7 @@
         </is>
       </c>
       <c r="B23" s="21" t="n">
-        <v>0.2275</v>
+        <v>0.315</v>
       </c>
     </row>
     <row r="24">
@@ -1229,7 +1229,7 @@
         </is>
       </c>
       <c r="B25" s="21" t="n">
-        <v>0.315</v>
+        <v>0.2275</v>
       </c>
     </row>
     <row r="31">
@@ -1256,7 +1256,7 @@
         </is>
       </c>
       <c r="B33" s="21" t="n">
-        <v>0.2275</v>
+        <v>0.315</v>
       </c>
     </row>
     <row r="34">
@@ -1276,7 +1276,7 @@
         </is>
       </c>
       <c r="B35" s="21" t="n">
-        <v>0.315</v>
+        <v>0.2275</v>
       </c>
     </row>
   </sheetData>
@@ -1291,7 +1291,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1600,65 +1600,72 @@
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="4" t="inlineStr">
-        <is>
-          <t>Paper ledger mark-to-market (as of 2026-10-24)</t>
+    <row r="14">
+      <c r="A14" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="B14" s="23" t="n">
+        <v>0.0464</v>
+      </c>
+      <c r="C14" s="23" t="n">
+        <v>0.1689</v>
+      </c>
+      <c r="D14" s="13" t="inlineStr">
+        <is>
+          <t>REFLATION</t>
+        </is>
+      </c>
+      <c r="E14" s="13" t="inlineStr">
+        <is>
+          <t>REFLATION</t>
+        </is>
+      </c>
+      <c r="F14" s="13" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="9" t="inlineStr">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Paper ledger mark-to-market (as of 2026-10-31)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="9" t="inlineStr">
         <is>
           <t>Tier</t>
         </is>
       </c>
-      <c r="B17" s="9" t="inlineStr">
+      <c r="B18" s="9" t="inlineStr">
         <is>
           <t>Since</t>
         </is>
       </c>
-      <c r="C17" s="9" t="inlineStr">
+      <c r="C18" s="9" t="inlineStr">
         <is>
           <t>Return</t>
         </is>
       </c>
-      <c r="D17" s="9" t="inlineStr">
+      <c r="D18" s="9" t="inlineStr">
         <is>
           <t>Max drawdown</t>
         </is>
       </c>
-      <c r="E17" s="9" t="inlineStr">
+      <c r="E18" s="9" t="inlineStr">
         <is>
           <t>Trading days</t>
         </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="13" t="inlineStr">
-        <is>
-          <t>CONS</t>
-        </is>
-      </c>
-      <c r="B18" s="13" t="inlineStr">
-        <is>
-          <t>2026-08-20</t>
-        </is>
-      </c>
-      <c r="C18" s="24" t="n">
-        <v>0.01732079494266392</v>
-      </c>
-      <c r="D18" s="24" t="n">
-        <v>-0.02204984823786937</v>
-      </c>
-      <c r="E18" s="13" t="n">
-        <v>45</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="13" t="inlineStr">
         <is>
-          <t>MOD</t>
+          <t>CONS</t>
         </is>
       </c>
       <c r="B19" s="13" t="inlineStr">
@@ -1667,19 +1674,19 @@
         </is>
       </c>
       <c r="C19" s="24" t="n">
-        <v>0.02478359698872024</v>
+        <v>0.01207834688351483</v>
       </c>
       <c r="D19" s="24" t="n">
-        <v>-0.03063726832854285</v>
+        <v>-0.02204984823786937</v>
       </c>
       <c r="E19" s="13" t="n">
-        <v>45</v>
+        <v>50</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="13" t="inlineStr">
         <is>
-          <t>AGG</t>
+          <t>MOD</t>
         </is>
       </c>
       <c r="B20" s="13" t="inlineStr">
@@ -1688,19 +1695,19 @@
         </is>
       </c>
       <c r="C20" s="24" t="n">
-        <v>0.04366982008972542</v>
+        <v>0.01616269649527879</v>
       </c>
       <c r="D20" s="24" t="n">
-        <v>-0.02704464641821624</v>
+        <v>-0.03063726832854285</v>
       </c>
       <c r="E20" s="13" t="n">
-        <v>45</v>
+        <v>50</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="13" t="inlineStr">
         <is>
-          <t>VAGG</t>
+          <t>AGG</t>
         </is>
       </c>
       <c r="B21" s="13" t="inlineStr">
@@ -1709,38 +1716,59 @@
         </is>
       </c>
       <c r="C21" s="24" t="n">
-        <v>0.008901791907482304</v>
+        <v>0.03123684706968444</v>
       </c>
       <c r="D21" s="24" t="n">
-        <v>-0.05516467405412073</v>
+        <v>-0.02704464641821624</v>
       </c>
       <c r="E21" s="13" t="n">
-        <v>45</v>
+        <v>50</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="13" t="inlineStr">
         <is>
+          <t>VAGG</t>
+        </is>
+      </c>
+      <c r="B22" s="13" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="C22" s="24" t="n">
+        <v>-0.01549360903668751</v>
+      </c>
+      <c r="D22" s="24" t="n">
+        <v>-0.06526454191042841</v>
+      </c>
+      <c r="E22" s="13" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="13" t="inlineStr">
+        <is>
           <t>SPY (bench)</t>
         </is>
       </c>
-      <c r="B22" s="13" t="inlineStr">
+      <c r="B23" s="13" t="inlineStr">
         <is>
           <t>2026-08-20</t>
         </is>
       </c>
-      <c r="C22" s="24" t="n">
-        <v>-0.0009741253031163577</v>
-      </c>
-      <c r="D22" s="24" t="n">
-        <v>-0.02472935182691627</v>
-      </c>
-      <c r="E22" s="13" t="n">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="8" t="inlineStr">
+      <c r="C23" s="24" t="n">
+        <v>-0.006561003905087182</v>
+      </c>
+      <c r="D23" s="24" t="n">
+        <v>-0.02999660545863914</v>
+      </c>
+      <c r="E23" s="13" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="8" t="inlineStr">
         <is>
           <t>Daily-rebalanced paper books from each ledger row's logged_at; SPY = buy-and-hold benchmark.</t>
         </is>

</xml_diff>

<commit_message>
Order workbook: per-month paper-book table on the Weekly Watch tab; regenerated on the November book at $17,500
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BBnnwzPLx94vYYG3d4vP48
</commit_message>
<xml_diff>
--- a/RotationOrders.xlsx
+++ b/RotationOrders.xlsx
@@ -1291,7 +1291,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F24"/>
+  <dimension ref="A1:H30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1300,6 +1300,8 @@
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1774,6 +1776,151 @@
         </is>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Paper books by ledger month (books as logged, held over each row's window)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="9" t="inlineStr">
+        <is>
+          <t>Month</t>
+        </is>
+      </c>
+      <c r="B27" s="9" t="inlineStr">
+        <is>
+          <t>Quadrant</t>
+        </is>
+      </c>
+      <c r="C27" s="9" t="inlineStr">
+        <is>
+          <t>CONS</t>
+        </is>
+      </c>
+      <c r="D27" s="9" t="inlineStr">
+        <is>
+          <t>MOD</t>
+        </is>
+      </c>
+      <c r="E27" s="9" t="inlineStr">
+        <is>
+          <t>AGG</t>
+        </is>
+      </c>
+      <c r="F27" s="9" t="inlineStr">
+        <is>
+          <t>VAGG</t>
+        </is>
+      </c>
+      <c r="G27" s="9" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="H27" s="9" t="inlineStr">
+        <is>
+          <t>Window</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="13" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B28" s="13" t="inlineStr">
+        <is>
+          <t>REFLATION</t>
+        </is>
+      </c>
+      <c r="C28" s="24" t="n">
+        <v>-0.002104323627920013</v>
+      </c>
+      <c r="D28" s="24" t="n">
+        <v>-0.002065329230729662</v>
+      </c>
+      <c r="E28" s="24" t="n">
+        <v>-0.006677854169061526</v>
+      </c>
+      <c r="F28" s="24" t="n">
+        <v>-0.005248806642418558</v>
+      </c>
+      <c r="G28" s="24" t="n">
+        <v>-0.00107522059031806</v>
+      </c>
+      <c r="H28" s="13" t="inlineStr">
+        <is>
+          <t>2026-08-21 to 2026-09-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="13" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="B29" s="13" t="inlineStr">
+        <is>
+          <t>REFLATION</t>
+        </is>
+      </c>
+      <c r="C29" s="24" t="n">
+        <v>-0.00168026014317646</v>
+      </c>
+      <c r="D29" s="24" t="n">
+        <v>-0.001199128555264939</v>
+      </c>
+      <c r="E29" s="24" t="n">
+        <v>0.01783767736803599</v>
+      </c>
+      <c r="F29" s="24" t="n">
+        <v>0.01607243431396155</v>
+      </c>
+      <c r="G29" s="24" t="n">
+        <v>0.005391447835549901</v>
+      </c>
+      <c r="H29" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-02 to 2026-10-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="13" t="inlineStr">
+        <is>
+          <t>2026-10</t>
+        </is>
+      </c>
+      <c r="B30" s="13" t="inlineStr">
+        <is>
+          <t>REFLATION</t>
+        </is>
+      </c>
+      <c r="C30" s="24" t="n">
+        <v>0.01591958756758638</v>
+      </c>
+      <c r="D30" s="24" t="n">
+        <v>0.01948824798438231</v>
+      </c>
+      <c r="E30" s="24" t="n">
+        <v>0.01997559659390014</v>
+      </c>
+      <c r="F30" s="24" t="n">
+        <v>-0.02595414710385879</v>
+      </c>
+      <c r="G30" s="24" t="n">
+        <v>-0.01082477471820464</v>
+      </c>
+      <c r="H30" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-02 to 2026-10-30</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>